<commit_message>
added excel files folder
</commit_message>
<xml_diff>
--- a/TCPL Rulesets - GL1 (1).xlsx
+++ b/TCPL Rulesets - GL1 (1).xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29127"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
   <workbookPr codeName="ThisWorkbook" defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\SEM-8\Data Rules Set Check\Data_rulesets_check\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\SW526XH\Downloads\Data Quality Check\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2A1D9F45-8178-426E-B307-EEB069DA8D87}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{954E4218-E8A8-4269-9539-16B5C55279DE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" tabRatio="906" firstSheet="2" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11020" tabRatio="906" firstSheet="2" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Data Availability backup" sheetId="89" state="hidden" r:id="rId1"/>
@@ -75,21 +75,21 @@
 </file>
 
 <file path=xl/metadata.xml><?xml version="1.0" encoding="utf-8"?>
-<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xlrd="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata">
   <metadataTypes count="1">
     <metadataType name="XLRICHVALUE" minSupportedVersion="120000" copy="1" pasteAll="1" pasteValues="1" merge="1" splitFirst="1" rowColShift="1" clearFormats="1" clearComments="1" assign="1" coerce="1"/>
   </metadataTypes>
   <futureMetadata name="XLRICHVALUE" count="2">
     <bk>
       <extLst>
-        <ext xmlns:xlrd="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata" uri="{3e2802c4-a4d2-4d8b-9148-e3be6c30e623}">
+        <ext uri="{3e2802c4-a4d2-4d8b-9148-e3be6c30e623}">
           <xlrd:rvb i="0"/>
         </ext>
       </extLst>
     </bk>
     <bk>
       <extLst>
-        <ext xmlns:xlrd="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata" uri="{3e2802c4-a4d2-4d8b-9148-e3be6c30e623}">
+        <ext uri="{3e2802c4-a4d2-4d8b-9148-e3be6c30e623}">
           <xlrd:rvb i="1"/>
         </ext>
       </extLst>
@@ -1280,10 +1280,6 @@
   </si>
   <si>
     <t>CompanyCode</t>
-  </si>
-  <si>
-    <t>1. Field should be 1001 / 1006 / 1009
-2.Field should not be blank</t>
   </si>
   <si>
     <t>Production Plant</t>
@@ -2535,6 +2531,9 @@
   </si>
   <si>
     <t>DisplayValue</t>
+  </si>
+  <si>
+    <t>1. Field should be 1001 / 1006 / 1009 2.Field should not be blank</t>
   </si>
 </sst>
 </file>
@@ -5498,9 +5497,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - 2022 Theme">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2013 - 2022">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -5538,7 +5537,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2013 - 2022">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -5644,7 +5643,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2013 - 2022">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -5786,7 +5785,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -7193,7 +7192,7 @@
     </row>
     <row r="2" spans="1:9" ht="26.15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B2" s="193" t="s">
-        <v>497</v>
+        <v>496</v>
       </c>
       <c r="C2" s="194"/>
       <c r="D2" s="170"/>
@@ -7216,7 +7215,7 @@
     </row>
     <row r="5" spans="1:9" ht="26.15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A5" s="181" t="s">
-        <v>498</v>
+        <v>497</v>
       </c>
       <c r="B5" s="181"/>
       <c r="C5" s="181"/>
@@ -7228,7 +7227,7 @@
     </row>
     <row r="6" spans="1:9" ht="32.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A6" s="195" t="s">
-        <v>499</v>
+        <v>498</v>
       </c>
       <c r="B6" s="195"/>
       <c r="C6" s="195"/>
@@ -7253,7 +7252,7 @@
         <v>295</v>
       </c>
       <c r="E7" s="47" t="s">
-        <v>500</v>
+        <v>499</v>
       </c>
       <c r="F7" s="47" t="s">
         <v>234</v>
@@ -7270,22 +7269,22 @@
     </row>
     <row r="8" spans="1:9" ht="29" x14ac:dyDescent="0.35">
       <c r="A8" s="6" t="s">
+        <v>500</v>
+      </c>
+      <c r="B8" s="6" t="s">
         <v>501</v>
       </c>
-      <c r="B8" s="6" t="s">
+      <c r="C8" s="8" t="s">
         <v>502</v>
-      </c>
-      <c r="C8" s="8" t="s">
-        <v>503</v>
       </c>
       <c r="D8" s="6" t="s">
         <v>235</v>
       </c>
       <c r="E8" s="106" t="s">
-        <v>463</v>
+        <v>462</v>
       </c>
       <c r="F8" s="106" t="s">
-        <v>463</v>
+        <v>462</v>
       </c>
       <c r="G8" s="26" t="s">
         <v>312</v>
@@ -7297,22 +7296,22 @@
     </row>
     <row r="9" spans="1:9" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A9" s="6" t="s">
+        <v>503</v>
+      </c>
+      <c r="B9" s="120" t="s">
         <v>504</v>
       </c>
-      <c r="B9" s="120" t="s">
+      <c r="C9" s="8" t="s">
         <v>505</v>
-      </c>
-      <c r="C9" s="8" t="s">
-        <v>506</v>
       </c>
       <c r="D9" s="6" t="s">
         <v>235</v>
       </c>
       <c r="E9" s="106" t="s">
-        <v>463</v>
+        <v>462</v>
       </c>
       <c r="F9" s="106" t="s">
-        <v>459</v>
+        <v>458</v>
       </c>
       <c r="G9" s="26" t="s">
         <v>312</v>
@@ -7324,25 +7323,25 @@
     </row>
     <row r="10" spans="1:9" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A10" s="6" t="s">
+        <v>506</v>
+      </c>
+      <c r="B10" s="120" t="s">
         <v>507</v>
       </c>
-      <c r="B10" s="120" t="s">
-        <v>508</v>
-      </c>
       <c r="C10" s="8" t="s">
-        <v>506</v>
+        <v>505</v>
       </c>
       <c r="D10" s="6" t="s">
         <v>235</v>
       </c>
       <c r="E10" s="106" t="s">
+        <v>462</v>
+      </c>
+      <c r="F10" s="106" t="s">
         <v>463</v>
       </c>
-      <c r="F10" s="106" t="s">
-        <v>464</v>
-      </c>
       <c r="G10" s="24" t="s">
-        <v>509</v>
+        <v>508</v>
       </c>
       <c r="H10" s="24" t="s">
         <v>308</v>
@@ -7351,20 +7350,20 @@
     </row>
     <row r="11" spans="1:9" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A11" s="6" t="s">
+        <v>509</v>
+      </c>
+      <c r="B11" s="120" t="s">
         <v>510</v>
       </c>
-      <c r="B11" s="120" t="s">
-        <v>511</v>
-      </c>
       <c r="C11" s="8" t="s">
-        <v>506</v>
+        <v>505</v>
       </c>
       <c r="D11" s="6"/>
       <c r="E11" s="106" t="s">
-        <v>459</v>
+        <v>458</v>
       </c>
       <c r="F11" s="106" t="s">
-        <v>512</v>
+        <v>511</v>
       </c>
       <c r="G11" s="26" t="s">
         <v>312</v>
@@ -7376,23 +7375,23 @@
     </row>
     <row r="12" spans="1:9" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A12" s="6" t="s">
+        <v>512</v>
+      </c>
+      <c r="B12" s="120" t="s">
         <v>513</v>
       </c>
-      <c r="B12" s="120" t="s">
+      <c r="C12" s="6" t="s">
         <v>514</v>
-      </c>
-      <c r="C12" s="6" t="s">
-        <v>515</v>
       </c>
       <c r="D12" s="6"/>
       <c r="E12" s="106" t="s">
+        <v>458</v>
+      </c>
+      <c r="F12" s="106" t="s">
         <v>459</v>
       </c>
-      <c r="F12" s="106" t="s">
-        <v>460</v>
-      </c>
       <c r="G12" s="145" t="s">
-        <v>516</v>
+        <v>515</v>
       </c>
       <c r="H12" s="24" t="s">
         <v>308</v>
@@ -7401,20 +7400,20 @@
     </row>
     <row r="13" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A13" s="6" t="s">
+        <v>516</v>
+      </c>
+      <c r="B13" s="6" t="s">
         <v>517</v>
       </c>
-      <c r="B13" s="6" t="s">
+      <c r="C13" s="8" t="s">
         <v>518</v>
-      </c>
-      <c r="C13" s="8" t="s">
-        <v>519</v>
       </c>
       <c r="D13" s="6"/>
       <c r="E13" s="106" t="s">
+        <v>519</v>
+      </c>
+      <c r="F13" s="106" t="s">
         <v>520</v>
-      </c>
-      <c r="F13" s="106" t="s">
-        <v>521</v>
       </c>
       <c r="G13" s="26" t="s">
         <v>312</v>
@@ -7426,13 +7425,13 @@
     </row>
     <row r="14" spans="1:9" ht="145" x14ac:dyDescent="0.35">
       <c r="A14" s="6" t="s">
-        <v>522</v>
+        <v>521</v>
       </c>
       <c r="B14" s="8" t="s">
         <v>26</v>
       </c>
       <c r="C14" s="8" t="s">
-        <v>523</v>
+        <v>522</v>
       </c>
       <c r="D14" s="6"/>
       <c r="E14" s="106" t="s">
@@ -7451,13 +7450,13 @@
     </row>
     <row r="15" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A15" s="6" t="s">
-        <v>524</v>
+        <v>523</v>
       </c>
       <c r="B15" s="6" t="s">
         <v>58</v>
       </c>
       <c r="C15" s="6" t="s">
-        <v>525</v>
+        <v>524</v>
       </c>
       <c r="D15" s="6"/>
       <c r="E15" s="106" t="s">
@@ -7476,23 +7475,23 @@
     </row>
     <row r="16" spans="1:9" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A16" s="6" t="s">
+        <v>525</v>
+      </c>
+      <c r="B16" s="120" t="s">
         <v>526</v>
       </c>
-      <c r="B16" s="120" t="s">
+      <c r="C16" s="8" t="s">
         <v>527</v>
-      </c>
-      <c r="C16" s="8" t="s">
-        <v>528</v>
       </c>
       <c r="D16" s="6"/>
       <c r="E16" s="106" t="s">
-        <v>463</v>
+        <v>462</v>
       </c>
       <c r="F16" s="16" t="s">
-        <v>465</v>
+        <v>464</v>
       </c>
       <c r="G16" s="24" t="s">
-        <v>529</v>
+        <v>528</v>
       </c>
       <c r="H16" s="24" t="s">
         <v>308</v>
@@ -7501,23 +7500,23 @@
     </row>
     <row r="17" spans="1:9" ht="29" x14ac:dyDescent="0.35">
       <c r="A17" s="6" t="s">
+        <v>529</v>
+      </c>
+      <c r="B17" s="120" t="s">
         <v>530</v>
       </c>
-      <c r="B17" s="120" t="s">
+      <c r="C17" s="8" t="s">
         <v>531</v>
-      </c>
-      <c r="C17" s="8" t="s">
-        <v>532</v>
       </c>
       <c r="D17" s="6"/>
       <c r="E17" s="106" t="s">
+        <v>462</v>
+      </c>
+      <c r="F17" s="16" t="s">
         <v>463</v>
       </c>
-      <c r="F17" s="16" t="s">
-        <v>464</v>
-      </c>
       <c r="G17" s="24" t="s">
-        <v>533</v>
+        <v>532</v>
       </c>
       <c r="H17" s="24" t="s">
         <v>308</v>
@@ -7526,20 +7525,20 @@
     </row>
     <row r="18" spans="1:9" ht="29" x14ac:dyDescent="0.35">
       <c r="A18" s="6" t="s">
+        <v>533</v>
+      </c>
+      <c r="B18" s="6" t="s">
         <v>534</v>
       </c>
-      <c r="B18" s="6" t="s">
+      <c r="C18" s="8" t="s">
         <v>535</v>
-      </c>
-      <c r="C18" s="8" t="s">
-        <v>536</v>
       </c>
       <c r="D18" s="6"/>
       <c r="E18" s="107" t="s">
-        <v>520</v>
+        <v>519</v>
       </c>
       <c r="F18" s="16" t="s">
-        <v>537</v>
+        <v>536</v>
       </c>
       <c r="G18" s="26" t="s">
         <v>312</v>
@@ -7551,20 +7550,20 @@
     </row>
     <row r="19" spans="1:9" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A19" s="6" t="s">
-        <v>538</v>
+        <v>537</v>
       </c>
       <c r="B19" s="6" t="s">
         <v>59</v>
       </c>
       <c r="C19" s="8" t="s">
-        <v>539</v>
+        <v>538</v>
       </c>
       <c r="D19" s="6"/>
       <c r="E19" s="106" t="s">
-        <v>463</v>
+        <v>462</v>
       </c>
       <c r="F19" s="16" t="s">
-        <v>540</v>
+        <v>539</v>
       </c>
       <c r="G19" s="26" t="s">
         <v>312</v>
@@ -7576,20 +7575,20 @@
     </row>
     <row r="20" spans="1:9" ht="41.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A20" s="6" t="s">
+        <v>540</v>
+      </c>
+      <c r="B20" s="6" t="s">
         <v>541</v>
       </c>
-      <c r="B20" s="6" t="s">
+      <c r="C20" s="8" t="s">
         <v>542</v>
-      </c>
-      <c r="C20" s="8" t="s">
-        <v>543</v>
       </c>
       <c r="D20" s="6"/>
       <c r="E20" s="106" t="s">
-        <v>463</v>
+        <v>462</v>
       </c>
       <c r="F20" s="16" t="s">
-        <v>544</v>
+        <v>543</v>
       </c>
       <c r="G20" s="26" t="s">
         <v>312</v>
@@ -7601,13 +7600,13 @@
     </row>
     <row r="21" spans="1:9" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A21" s="6" t="s">
+        <v>544</v>
+      </c>
+      <c r="B21" s="120" t="s">
         <v>545</v>
       </c>
-      <c r="B21" s="120" t="s">
+      <c r="C21" s="8" t="s">
         <v>546</v>
-      </c>
-      <c r="C21" s="8" t="s">
-        <v>547</v>
       </c>
       <c r="D21" s="6"/>
       <c r="E21" s="106" t="s">
@@ -7629,7 +7628,7 @@
     </row>
     <row r="23" spans="1:9" x14ac:dyDescent="0.3">
       <c r="B23" s="35" t="s">
-        <v>548</v>
+        <v>547</v>
       </c>
       <c r="F23" s="61"/>
     </row>
@@ -7639,7 +7638,7 @@
       <selection activeCell="H4" sqref="H4:J11"/>
       <pageMargins left="0" right="0" top="0" bottom="0" header="0" footer="0"/>
       <pageSetup orientation="portrait" r:id="rId1"/>
-      <autoFilter ref="A2:O16" xr:uid="{8095BEDC-A695-4DDC-A442-DFE8BA62A908}">
+      <autoFilter ref="A2:O16" xr:uid="{9C1F0F38-FB03-4A75-8325-9FA0BD6F4877}">
         <filterColumn colId="11">
           <filters>
             <filter val="No"/>
@@ -7694,7 +7693,7 @@
     </row>
     <row r="2" spans="1:9" ht="39.65" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B2" s="196" t="s">
-        <v>549</v>
+        <v>548</v>
       </c>
       <c r="C2" s="197"/>
       <c r="D2" s="173"/>
@@ -7717,7 +7716,7 @@
     </row>
     <row r="5" spans="1:9" ht="39.65" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A5" s="198" t="s">
-        <v>550</v>
+        <v>549</v>
       </c>
       <c r="B5" s="199"/>
       <c r="C5" s="199"/>
@@ -7730,7 +7729,7 @@
     </row>
     <row r="6" spans="1:9" ht="39.65" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A6" s="201" t="s">
-        <v>551</v>
+        <v>550</v>
       </c>
       <c r="B6" s="202"/>
       <c r="C6" s="202"/>
@@ -7772,25 +7771,25 @@
     </row>
     <row r="8" spans="1:9" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A8" s="6" t="s">
+        <v>551</v>
+      </c>
+      <c r="B8" s="8" t="s">
         <v>552</v>
       </c>
-      <c r="B8" s="8" t="s">
+      <c r="C8" s="8" t="s">
         <v>553</v>
-      </c>
-      <c r="C8" s="8" t="s">
-        <v>554</v>
       </c>
       <c r="D8" s="6" t="s">
         <v>235</v>
       </c>
       <c r="E8" s="106" t="s">
+        <v>554</v>
+      </c>
+      <c r="F8" s="106" t="s">
         <v>555</v>
       </c>
-      <c r="F8" s="106" t="s">
-        <v>556</v>
-      </c>
       <c r="G8" s="24" t="s">
-        <v>529</v>
+        <v>528</v>
       </c>
       <c r="H8" s="24" t="s">
         <v>308</v>
@@ -7799,25 +7798,25 @@
     </row>
     <row r="9" spans="1:9" ht="29" x14ac:dyDescent="0.35">
       <c r="A9" s="6" t="s">
-        <v>557</v>
+        <v>556</v>
       </c>
       <c r="B9" s="8" t="s">
         <v>238</v>
       </c>
       <c r="C9" s="8" t="s">
-        <v>558</v>
+        <v>557</v>
       </c>
       <c r="D9" s="6" t="s">
         <v>235</v>
       </c>
       <c r="E9" s="106" t="s">
-        <v>555</v>
+        <v>554</v>
       </c>
       <c r="F9" s="106" t="s">
         <v>43</v>
       </c>
       <c r="G9" s="24" t="s">
-        <v>533</v>
+        <v>532</v>
       </c>
       <c r="H9" s="24" t="s">
         <v>308</v>
@@ -7826,25 +7825,25 @@
     </row>
     <row r="10" spans="1:9" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A10" s="6" t="s">
-        <v>559</v>
+        <v>558</v>
       </c>
       <c r="B10" s="8" t="s">
         <v>182</v>
       </c>
       <c r="C10" s="8" t="s">
-        <v>560</v>
+        <v>559</v>
       </c>
       <c r="D10" s="6" t="s">
         <v>235</v>
       </c>
       <c r="E10" s="106" t="s">
+        <v>560</v>
+      </c>
+      <c r="F10" s="106" t="s">
         <v>561</v>
       </c>
-      <c r="F10" s="106" t="s">
-        <v>562</v>
-      </c>
       <c r="G10" s="56" t="s">
-        <v>516</v>
+        <v>515</v>
       </c>
       <c r="H10" s="24" t="s">
         <v>308</v>
@@ -7853,25 +7852,25 @@
     </row>
     <row r="11" spans="1:9" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A11" s="6" t="s">
+        <v>562</v>
+      </c>
+      <c r="B11" s="122" t="s">
         <v>563</v>
       </c>
-      <c r="B11" s="122" t="s">
+      <c r="C11" s="59" t="s">
         <v>564</v>
-      </c>
-      <c r="C11" s="59" t="s">
-        <v>565</v>
       </c>
       <c r="D11" s="6" t="s">
         <v>235</v>
       </c>
       <c r="E11" s="106" t="s">
-        <v>561</v>
+        <v>560</v>
       </c>
       <c r="F11" s="106" t="s">
+        <v>565</v>
+      </c>
+      <c r="G11" s="24" t="s">
         <v>566</v>
-      </c>
-      <c r="G11" s="24" t="s">
-        <v>567</v>
       </c>
       <c r="H11" s="24" t="s">
         <v>302</v>
@@ -7880,7 +7879,7 @@
     </row>
     <row r="14" spans="1:9" x14ac:dyDescent="0.35">
       <c r="B14" t="s">
-        <v>568</v>
+        <v>567</v>
       </c>
     </row>
   </sheetData>
@@ -7931,7 +7930,7 @@
     </row>
     <row r="2" spans="1:9" ht="39.65" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B2" s="196" t="s">
-        <v>549</v>
+        <v>548</v>
       </c>
       <c r="C2" s="197"/>
       <c r="D2" s="173"/>
@@ -7954,7 +7953,7 @@
     </row>
     <row r="5" spans="1:9" ht="39.65" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A5" s="198" t="s">
-        <v>569</v>
+        <v>568</v>
       </c>
       <c r="B5" s="199"/>
       <c r="C5" s="199"/>
@@ -7966,7 +7965,7 @@
     </row>
     <row r="6" spans="1:9" ht="39.65" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A6" s="186" t="s">
-        <v>570</v>
+        <v>569</v>
       </c>
       <c r="B6" s="186"/>
       <c r="C6" s="186"/>
@@ -8007,25 +8006,25 @@
     </row>
     <row r="8" spans="1:9" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A8" s="6" t="s">
-        <v>571</v>
+        <v>570</v>
       </c>
       <c r="B8" s="8" t="s">
+        <v>552</v>
+      </c>
+      <c r="C8" s="8" t="s">
         <v>553</v>
-      </c>
-      <c r="C8" s="8" t="s">
-        <v>554</v>
       </c>
       <c r="D8" s="6" t="s">
         <v>235</v>
       </c>
       <c r="E8" s="6" t="s">
+        <v>554</v>
+      </c>
+      <c r="F8" s="106" t="s">
         <v>555</v>
       </c>
-      <c r="F8" s="106" t="s">
-        <v>556</v>
-      </c>
       <c r="G8" s="24" t="s">
-        <v>529</v>
+        <v>528</v>
       </c>
       <c r="H8" s="24" t="s">
         <v>308</v>
@@ -8034,25 +8033,25 @@
     </row>
     <row r="9" spans="1:9" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A9" s="6" t="s">
-        <v>572</v>
+        <v>571</v>
       </c>
       <c r="B9" s="8" t="s">
         <v>238</v>
       </c>
       <c r="C9" s="8" t="s">
-        <v>558</v>
+        <v>557</v>
       </c>
       <c r="D9" s="6" t="s">
         <v>235</v>
       </c>
       <c r="E9" s="6" t="s">
-        <v>555</v>
+        <v>554</v>
       </c>
       <c r="F9" s="106" t="s">
         <v>43</v>
       </c>
       <c r="G9" s="24" t="s">
-        <v>533</v>
+        <v>532</v>
       </c>
       <c r="H9" s="24" t="s">
         <v>308</v>
@@ -8061,25 +8060,25 @@
     </row>
     <row r="10" spans="1:9" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A10" s="6" t="s">
-        <v>573</v>
+        <v>572</v>
       </c>
       <c r="B10" s="8" t="s">
         <v>182</v>
       </c>
       <c r="C10" s="8" t="s">
-        <v>560</v>
+        <v>559</v>
       </c>
       <c r="D10" s="6" t="s">
         <v>235</v>
       </c>
       <c r="E10" s="6" t="s">
-        <v>574</v>
+        <v>573</v>
       </c>
       <c r="F10" s="106" t="s">
-        <v>562</v>
+        <v>561</v>
       </c>
       <c r="G10" s="56" t="s">
-        <v>516</v>
+        <v>515</v>
       </c>
       <c r="H10" s="24" t="s">
         <v>308</v>
@@ -8088,25 +8087,25 @@
     </row>
     <row r="11" spans="1:9" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A11" s="6" t="s">
-        <v>575</v>
+        <v>574</v>
       </c>
       <c r="B11" s="122" t="s">
+        <v>563</v>
+      </c>
+      <c r="C11" s="59" t="s">
         <v>564</v>
-      </c>
-      <c r="C11" s="59" t="s">
-        <v>565</v>
       </c>
       <c r="D11" s="6" t="s">
         <v>235</v>
       </c>
       <c r="E11" s="6" t="s">
-        <v>574</v>
+        <v>573</v>
       </c>
       <c r="F11" s="106" t="s">
+        <v>565</v>
+      </c>
+      <c r="G11" s="24" t="s">
         <v>566</v>
-      </c>
-      <c r="G11" s="24" t="s">
-        <v>567</v>
       </c>
       <c r="H11" s="24" t="s">
         <v>302</v>
@@ -8159,7 +8158,7 @@
     </row>
     <row r="2" spans="1:8" ht="34.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B2" s="204" t="s">
-        <v>576</v>
+        <v>575</v>
       </c>
       <c r="C2" s="205"/>
       <c r="D2" s="173"/>
@@ -8179,7 +8178,7 @@
     </row>
     <row r="5" spans="1:8" ht="34.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A5" s="170" t="s">
-        <v>577</v>
+        <v>576</v>
       </c>
       <c r="B5" s="170"/>
       <c r="C5" s="170"/>
@@ -8191,7 +8190,7 @@
     </row>
     <row r="6" spans="1:8" ht="29.15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A6" s="169" t="s">
-        <v>578</v>
+        <v>577</v>
       </c>
       <c r="B6" s="169"/>
       <c r="C6" s="169"/>
@@ -8229,13 +8228,13 @@
     </row>
     <row r="8" spans="1:8" ht="29" x14ac:dyDescent="0.35">
       <c r="A8" s="6" t="s">
+        <v>578</v>
+      </c>
+      <c r="B8" s="6" t="s">
+        <v>552</v>
+      </c>
+      <c r="C8" s="6" t="s">
         <v>579</v>
-      </c>
-      <c r="B8" s="6" t="s">
-        <v>553</v>
-      </c>
-      <c r="C8" s="6" t="s">
-        <v>580</v>
       </c>
       <c r="D8" s="6" t="s">
         <v>276</v>
@@ -8244,33 +8243,33 @@
         <v>82</v>
       </c>
       <c r="F8" s="24" t="s">
-        <v>581</v>
+        <v>580</v>
       </c>
       <c r="G8" s="72" t="s">
         <v>302</v>
       </c>
       <c r="H8" s="8" t="s">
-        <v>582</v>
+        <v>581</v>
       </c>
     </row>
     <row r="9" spans="1:8" ht="29" x14ac:dyDescent="0.35">
       <c r="A9" s="6" t="s">
-        <v>583</v>
+        <v>582</v>
       </c>
       <c r="B9" s="6" t="s">
         <v>240</v>
       </c>
       <c r="C9" s="6" t="s">
-        <v>584</v>
+        <v>583</v>
       </c>
       <c r="D9" s="6" t="s">
         <v>243</v>
       </c>
       <c r="E9" s="6" t="s">
-        <v>585</v>
+        <v>584</v>
       </c>
       <c r="F9" s="24" t="s">
-        <v>581</v>
+        <v>580</v>
       </c>
       <c r="G9" s="72" t="s">
         <v>302</v>
@@ -8279,20 +8278,20 @@
     </row>
     <row r="10" spans="1:8" ht="29" x14ac:dyDescent="0.35">
       <c r="A10" s="6" t="s">
-        <v>586</v>
+        <v>585</v>
       </c>
       <c r="B10" s="6" t="s">
         <v>74</v>
       </c>
       <c r="C10" s="6"/>
       <c r="D10" s="6" t="s">
+        <v>586</v>
+      </c>
+      <c r="E10" s="6" t="s">
         <v>587</v>
       </c>
-      <c r="E10" s="6" t="s">
-        <v>588</v>
-      </c>
       <c r="F10" s="24" t="s">
-        <v>581</v>
+        <v>580</v>
       </c>
       <c r="G10" s="72" t="s">
         <v>302</v>
@@ -8301,20 +8300,20 @@
     </row>
     <row r="11" spans="1:8" ht="29" x14ac:dyDescent="0.35">
       <c r="A11" s="6" t="s">
-        <v>589</v>
+        <v>588</v>
       </c>
       <c r="B11" s="6" t="s">
         <v>75</v>
       </c>
       <c r="C11" s="6"/>
       <c r="D11" s="6" t="s">
+        <v>589</v>
+      </c>
+      <c r="E11" s="6" t="s">
         <v>590</v>
       </c>
-      <c r="E11" s="6" t="s">
-        <v>591</v>
-      </c>
       <c r="F11" s="24" t="s">
-        <v>581</v>
+        <v>580</v>
       </c>
       <c r="G11" s="72" t="s">
         <v>302</v>
@@ -8323,22 +8322,22 @@
     </row>
     <row r="12" spans="1:8" ht="29" x14ac:dyDescent="0.35">
       <c r="A12" s="6" t="s">
-        <v>592</v>
+        <v>591</v>
       </c>
       <c r="B12" s="153" t="s">
         <v>76</v>
       </c>
       <c r="C12" s="153" t="s">
+        <v>592</v>
+      </c>
+      <c r="D12" s="6" t="s">
         <v>593</v>
       </c>
-      <c r="D12" s="6" t="s">
-        <v>594</v>
-      </c>
       <c r="E12" s="153" t="s">
-        <v>427</v>
+        <v>426</v>
       </c>
       <c r="F12" s="24" t="s">
-        <v>581</v>
+        <v>580</v>
       </c>
       <c r="G12" s="72" t="s">
         <v>302</v>
@@ -8347,22 +8346,22 @@
     </row>
     <row r="13" spans="1:8" ht="29" x14ac:dyDescent="0.35">
       <c r="A13" s="6" t="s">
-        <v>595</v>
+        <v>594</v>
       </c>
       <c r="B13" s="153" t="s">
         <v>78</v>
       </c>
       <c r="C13" s="153" t="s">
+        <v>595</v>
+      </c>
+      <c r="D13" s="154" t="s">
         <v>596</v>
       </c>
-      <c r="D13" s="154" t="s">
+      <c r="E13" s="6" t="s">
         <v>597</v>
       </c>
-      <c r="E13" s="6" t="s">
-        <v>598</v>
-      </c>
       <c r="F13" s="24" t="s">
-        <v>581</v>
+        <v>580</v>
       </c>
       <c r="G13" s="72" t="s">
         <v>302</v>
@@ -8371,22 +8370,22 @@
     </row>
     <row r="14" spans="1:8" ht="29" x14ac:dyDescent="0.35">
       <c r="A14" s="6" t="s">
-        <v>599</v>
+        <v>598</v>
       </c>
       <c r="B14" s="6" t="s">
         <v>79</v>
       </c>
       <c r="C14" s="6" t="s">
+        <v>599</v>
+      </c>
+      <c r="D14" s="6" t="s">
         <v>600</v>
       </c>
-      <c r="D14" s="6" t="s">
+      <c r="E14" s="6" t="s">
         <v>601</v>
       </c>
-      <c r="E14" s="6" t="s">
-        <v>602</v>
-      </c>
       <c r="F14" s="24" t="s">
-        <v>581</v>
+        <v>580</v>
       </c>
       <c r="G14" s="72" t="s">
         <v>302</v>
@@ -8395,22 +8394,22 @@
     </row>
     <row r="15" spans="1:8" ht="29" x14ac:dyDescent="0.35">
       <c r="A15" s="6" t="s">
-        <v>603</v>
+        <v>602</v>
       </c>
       <c r="B15" s="6" t="s">
         <v>81</v>
       </c>
       <c r="C15" s="6" t="s">
+        <v>603</v>
+      </c>
+      <c r="D15" s="6" t="s">
+        <v>600</v>
+      </c>
+      <c r="E15" s="6" t="s">
         <v>604</v>
       </c>
-      <c r="D15" s="6" t="s">
-        <v>601</v>
-      </c>
-      <c r="E15" s="6" t="s">
-        <v>605</v>
-      </c>
       <c r="F15" s="24" t="s">
-        <v>581</v>
+        <v>580</v>
       </c>
       <c r="G15" s="72" t="s">
         <v>302</v>
@@ -8419,22 +8418,22 @@
     </row>
     <row r="16" spans="1:8" ht="29" x14ac:dyDescent="0.35">
       <c r="A16" s="6" t="s">
-        <v>606</v>
+        <v>605</v>
       </c>
       <c r="B16" s="6" t="s">
         <v>82</v>
       </c>
       <c r="C16" s="122" t="s">
+        <v>606</v>
+      </c>
+      <c r="D16" s="6" t="s">
+        <v>600</v>
+      </c>
+      <c r="E16" s="6" t="s">
         <v>607</v>
       </c>
-      <c r="D16" s="6" t="s">
-        <v>601</v>
-      </c>
-      <c r="E16" s="6" t="s">
-        <v>608</v>
-      </c>
       <c r="F16" s="24" t="s">
-        <v>581</v>
+        <v>580</v>
       </c>
       <c r="G16" s="72" t="s">
         <v>302</v>
@@ -8443,22 +8442,22 @@
     </row>
     <row r="17" spans="1:8" ht="29" x14ac:dyDescent="0.35">
       <c r="A17" s="6" t="s">
-        <v>609</v>
+        <v>608</v>
       </c>
       <c r="B17" s="6" t="s">
         <v>84</v>
       </c>
       <c r="C17" s="122" t="s">
+        <v>609</v>
+      </c>
+      <c r="D17" s="6" t="s">
+        <v>600</v>
+      </c>
+      <c r="E17" s="6" t="s">
         <v>610</v>
       </c>
-      <c r="D17" s="6" t="s">
-        <v>601</v>
-      </c>
-      <c r="E17" s="6" t="s">
-        <v>611</v>
-      </c>
       <c r="F17" s="24" t="s">
-        <v>581</v>
+        <v>580</v>
       </c>
       <c r="G17" s="72" t="s">
         <v>302</v>
@@ -8467,20 +8466,20 @@
     </row>
     <row r="18" spans="1:8" ht="29" x14ac:dyDescent="0.35">
       <c r="A18" s="6" t="s">
-        <v>612</v>
+        <v>611</v>
       </c>
       <c r="B18" s="6" t="s">
         <v>85</v>
       </c>
       <c r="C18" s="122"/>
       <c r="D18" s="6" t="s">
-        <v>601</v>
+        <v>600</v>
       </c>
       <c r="E18" s="154" t="s">
-        <v>613</v>
+        <v>612</v>
       </c>
       <c r="F18" s="24" t="s">
-        <v>581</v>
+        <v>580</v>
       </c>
       <c r="G18" s="72" t="s">
         <v>302</v>
@@ -8489,20 +8488,20 @@
     </row>
     <row r="19" spans="1:8" ht="29" x14ac:dyDescent="0.35">
       <c r="A19" s="6" t="s">
-        <v>614</v>
+        <v>613</v>
       </c>
       <c r="B19" s="6" t="s">
         <v>86</v>
       </c>
       <c r="C19" s="122"/>
       <c r="D19" s="6" t="s">
-        <v>601</v>
+        <v>600</v>
       </c>
       <c r="E19" s="154" t="s">
-        <v>615</v>
+        <v>614</v>
       </c>
       <c r="F19" s="24" t="s">
-        <v>581</v>
+        <v>580</v>
       </c>
       <c r="G19" s="72" t="s">
         <v>302</v>
@@ -8511,22 +8510,22 @@
     </row>
     <row r="20" spans="1:8" ht="29" x14ac:dyDescent="0.35">
       <c r="A20" s="6" t="s">
-        <v>616</v>
+        <v>615</v>
       </c>
       <c r="B20" s="6" t="s">
         <v>87</v>
       </c>
       <c r="C20" s="122" t="s">
+        <v>616</v>
+      </c>
+      <c r="D20" s="6" t="s">
+        <v>600</v>
+      </c>
+      <c r="E20" s="6" t="s">
         <v>617</v>
       </c>
-      <c r="D20" s="6" t="s">
-        <v>601</v>
-      </c>
-      <c r="E20" s="6" t="s">
-        <v>618</v>
-      </c>
       <c r="F20" s="24" t="s">
-        <v>581</v>
+        <v>580</v>
       </c>
       <c r="G20" s="72" t="s">
         <v>302</v>
@@ -8535,22 +8534,22 @@
     </row>
     <row r="21" spans="1:8" ht="29" x14ac:dyDescent="0.35">
       <c r="A21" s="6" t="s">
-        <v>619</v>
+        <v>618</v>
       </c>
       <c r="B21" s="6" t="s">
         <v>89</v>
       </c>
       <c r="C21" s="122" t="s">
+        <v>619</v>
+      </c>
+      <c r="D21" s="6" t="s">
+        <v>600</v>
+      </c>
+      <c r="E21" s="6" t="s">
         <v>620</v>
       </c>
-      <c r="D21" s="6" t="s">
-        <v>601</v>
-      </c>
-      <c r="E21" s="6" t="s">
-        <v>621</v>
-      </c>
       <c r="F21" s="24" t="s">
-        <v>581</v>
+        <v>580</v>
       </c>
       <c r="G21" s="72" t="s">
         <v>302</v>
@@ -8559,22 +8558,22 @@
     </row>
     <row r="22" spans="1:8" ht="29" x14ac:dyDescent="0.35">
       <c r="A22" s="6" t="s">
-        <v>622</v>
+        <v>621</v>
       </c>
       <c r="B22" s="6" t="s">
         <v>90</v>
       </c>
       <c r="C22" s="122" t="s">
+        <v>622</v>
+      </c>
+      <c r="D22" s="6" t="s">
+        <v>600</v>
+      </c>
+      <c r="E22" s="6" t="s">
         <v>623</v>
       </c>
-      <c r="D22" s="6" t="s">
-        <v>601</v>
-      </c>
-      <c r="E22" s="6" t="s">
-        <v>624</v>
-      </c>
       <c r="F22" s="24" t="s">
-        <v>581</v>
+        <v>580</v>
       </c>
       <c r="G22" s="72" t="s">
         <v>302</v>
@@ -8583,22 +8582,22 @@
     </row>
     <row r="23" spans="1:8" ht="29" x14ac:dyDescent="0.35">
       <c r="A23" s="6" t="s">
-        <v>625</v>
+        <v>624</v>
       </c>
       <c r="B23" s="6" t="s">
         <v>91</v>
       </c>
       <c r="C23" s="122" t="s">
+        <v>625</v>
+      </c>
+      <c r="D23" s="6" t="s">
+        <v>600</v>
+      </c>
+      <c r="E23" s="6" t="s">
         <v>626</v>
       </c>
-      <c r="D23" s="6" t="s">
-        <v>601</v>
-      </c>
-      <c r="E23" s="6" t="s">
-        <v>627</v>
-      </c>
       <c r="F23" s="24" t="s">
-        <v>581</v>
+        <v>580</v>
       </c>
       <c r="G23" s="72" t="s">
         <v>302</v>
@@ -8607,22 +8606,22 @@
     </row>
     <row r="24" spans="1:8" ht="29" x14ac:dyDescent="0.35">
       <c r="A24" s="6" t="s">
+        <v>627</v>
+      </c>
+      <c r="B24" s="6" t="s">
         <v>628</v>
       </c>
-      <c r="B24" s="6" t="s">
+      <c r="C24" s="122" t="s">
         <v>629</v>
       </c>
-      <c r="C24" s="122" t="s">
+      <c r="D24" s="6" t="s">
+        <v>600</v>
+      </c>
+      <c r="E24" s="154" t="s">
         <v>630</v>
       </c>
-      <c r="D24" s="6" t="s">
-        <v>601</v>
-      </c>
-      <c r="E24" s="154" t="s">
-        <v>631</v>
-      </c>
       <c r="F24" s="24" t="s">
-        <v>581</v>
+        <v>580</v>
       </c>
       <c r="G24" s="72" t="s">
         <v>302</v>
@@ -8631,22 +8630,22 @@
     </row>
     <row r="25" spans="1:8" ht="29" x14ac:dyDescent="0.35">
       <c r="A25" s="6" t="s">
+        <v>631</v>
+      </c>
+      <c r="B25" s="6" t="s">
         <v>632</v>
-      </c>
-      <c r="B25" s="6" t="s">
-        <v>633</v>
       </c>
       <c r="C25" s="122" t="s">
         <v>240</v>
       </c>
       <c r="D25" s="6" t="s">
-        <v>601</v>
+        <v>600</v>
       </c>
       <c r="E25" s="154" t="s">
-        <v>634</v>
+        <v>633</v>
       </c>
       <c r="F25" s="24" t="s">
-        <v>581</v>
+        <v>580</v>
       </c>
       <c r="G25" s="72" t="s">
         <v>302</v>
@@ -8655,22 +8654,22 @@
     </row>
     <row r="26" spans="1:8" ht="29" x14ac:dyDescent="0.35">
       <c r="A26" s="6" t="s">
-        <v>635</v>
+        <v>634</v>
       </c>
       <c r="B26" s="6" t="s">
         <v>92</v>
       </c>
       <c r="C26" s="122" t="s">
+        <v>635</v>
+      </c>
+      <c r="D26" s="6" t="s">
+        <v>600</v>
+      </c>
+      <c r="E26" s="6" t="s">
         <v>636</v>
       </c>
-      <c r="D26" s="6" t="s">
-        <v>601</v>
-      </c>
-      <c r="E26" s="6" t="s">
-        <v>637</v>
-      </c>
       <c r="F26" s="24" t="s">
-        <v>581</v>
+        <v>580</v>
       </c>
       <c r="G26" s="72" t="s">
         <v>302</v>
@@ -8679,22 +8678,22 @@
     </row>
     <row r="27" spans="1:8" ht="29" x14ac:dyDescent="0.35">
       <c r="A27" s="6" t="s">
-        <v>638</v>
+        <v>637</v>
       </c>
       <c r="B27" s="6" t="s">
         <v>93</v>
       </c>
       <c r="C27" s="122" t="s">
+        <v>638</v>
+      </c>
+      <c r="D27" s="6" t="s">
+        <v>600</v>
+      </c>
+      <c r="E27" s="6" t="s">
         <v>639</v>
       </c>
-      <c r="D27" s="6" t="s">
-        <v>601</v>
-      </c>
-      <c r="E27" s="6" t="s">
-        <v>640</v>
-      </c>
       <c r="F27" s="24" t="s">
-        <v>581</v>
+        <v>580</v>
       </c>
       <c r="G27" s="72" t="s">
         <v>302</v>
@@ -8703,22 +8702,22 @@
     </row>
     <row r="28" spans="1:8" ht="29" x14ac:dyDescent="0.35">
       <c r="A28" s="6" t="s">
-        <v>641</v>
+        <v>640</v>
       </c>
       <c r="B28" s="6" t="s">
         <v>94</v>
       </c>
       <c r="C28" s="158" t="s">
+        <v>641</v>
+      </c>
+      <c r="D28" s="158" t="s">
         <v>642</v>
       </c>
-      <c r="D28" s="158" t="s">
+      <c r="E28" s="158" t="s">
         <v>643</v>
       </c>
-      <c r="E28" s="158" t="s">
-        <v>644</v>
-      </c>
       <c r="F28" s="163" t="s">
-        <v>581</v>
+        <v>580</v>
       </c>
       <c r="G28" s="164" t="s">
         <v>302</v>
@@ -8727,18 +8726,18 @@
     </row>
     <row r="29" spans="1:8" s="35" customFormat="1" ht="29" x14ac:dyDescent="0.35">
       <c r="A29" s="6" t="s">
+        <v>644</v>
+      </c>
+      <c r="B29" s="168" t="s">
         <v>645</v>
       </c>
-      <c r="B29" s="168" t="s">
+      <c r="C29" s="168" t="s">
         <v>646</v>
-      </c>
-      <c r="C29" s="168" t="s">
-        <v>647</v>
       </c>
       <c r="D29" s="6"/>
       <c r="E29" s="157"/>
       <c r="F29" s="163" t="s">
-        <v>581</v>
+        <v>580</v>
       </c>
       <c r="G29" s="164" t="s">
         <v>302</v>
@@ -8747,20 +8746,20 @@
     </row>
     <row r="30" spans="1:8" ht="29" x14ac:dyDescent="0.35">
       <c r="A30" s="6" t="s">
-        <v>648</v>
+        <v>647</v>
       </c>
       <c r="B30" s="157" t="s">
         <v>95</v>
       </c>
       <c r="C30" s="66"/>
       <c r="D30" s="66" t="s">
-        <v>643</v>
+        <v>642</v>
       </c>
       <c r="E30" s="66" t="s">
-        <v>649</v>
+        <v>648</v>
       </c>
       <c r="F30" s="159" t="s">
-        <v>581</v>
+        <v>580</v>
       </c>
       <c r="G30" s="160" t="s">
         <v>302</v>
@@ -8769,16 +8768,16 @@
     </row>
     <row r="31" spans="1:8" ht="29" x14ac:dyDescent="0.35">
       <c r="A31" s="6" t="s">
+        <v>649</v>
+      </c>
+      <c r="B31" s="162" t="s">
         <v>650</v>
-      </c>
-      <c r="B31" s="162" t="s">
-        <v>651</v>
       </c>
       <c r="C31" s="66"/>
       <c r="D31" s="66"/>
       <c r="E31" s="66"/>
       <c r="F31" s="165" t="s">
-        <v>652</v>
+        <v>651</v>
       </c>
       <c r="G31" s="160" t="s">
         <v>302</v>
@@ -8787,7 +8786,7 @@
     </row>
     <row r="32" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A32" s="6" t="s">
-        <v>653</v>
+        <v>652</v>
       </c>
       <c r="B32" s="162" t="s">
         <v>332</v>
@@ -8869,7 +8868,7 @@
     </row>
     <row r="2" spans="1:7" ht="45.65" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A2" s="206" t="s">
-        <v>654</v>
+        <v>653</v>
       </c>
       <c r="B2" s="206"/>
       <c r="C2" s="173"/>
@@ -8894,10 +8893,10 @@
         <v>295</v>
       </c>
       <c r="D4" s="75" t="s">
+        <v>654</v>
+      </c>
+      <c r="E4" s="75" t="s">
         <v>655</v>
-      </c>
-      <c r="E4" s="75" t="s">
-        <v>656</v>
       </c>
       <c r="F4" s="116" t="s">
         <v>297</v>
@@ -8934,7 +8933,7 @@
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A7" s="21" t="s">
-        <v>657</v>
+        <v>656</v>
       </c>
       <c r="B7" s="5"/>
       <c r="C7" s="5"/>
@@ -8986,7 +8985,7 @@
     </row>
     <row r="2" spans="1:7" ht="46.4" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A2" s="182" t="s">
-        <v>658</v>
+        <v>657</v>
       </c>
       <c r="B2" s="182"/>
       <c r="C2" s="173"/>
@@ -9011,10 +9010,10 @@
         <v>295</v>
       </c>
       <c r="D4" s="75" t="s">
+        <v>654</v>
+      </c>
+      <c r="E4" s="75" t="s">
         <v>655</v>
-      </c>
-      <c r="E4" s="75" t="s">
-        <v>656</v>
       </c>
       <c r="F4" s="116" t="s">
         <v>297</v>
@@ -9025,7 +9024,7 @@
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A5" s="44" t="s">
-        <v>659</v>
+        <v>658</v>
       </c>
       <c r="B5" s="3"/>
       <c r="C5" s="3"/>
@@ -9051,7 +9050,7 @@
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A7" s="21" t="s">
-        <v>660</v>
+        <v>659</v>
       </c>
       <c r="B7" s="5"/>
       <c r="C7" s="3"/>
@@ -14801,7 +14800,7 @@
       <c r="E11" s="6"/>
       <c r="F11" s="6"/>
       <c r="G11" s="23" t="s">
-        <v>363</v>
+        <v>660</v>
       </c>
       <c r="H11" s="8" t="s">
         <v>308</v>
@@ -14811,53 +14810,53 @@
     <row r="12" spans="1:12" x14ac:dyDescent="0.35">
       <c r="C12" s="1"/>
       <c r="K12" s="118" t="s">
+        <v>363</v>
+      </c>
+      <c r="L12" s="119" t="s">
         <v>364</v>
-      </c>
-      <c r="L12" s="119" t="s">
-        <v>365</v>
       </c>
     </row>
     <row r="13" spans="1:12" x14ac:dyDescent="0.35">
       <c r="K13" s="11" t="s">
+        <v>365</v>
+      </c>
+      <c r="L13" s="12" t="s">
         <v>366</v>
-      </c>
-      <c r="L13" s="12" t="s">
-        <v>367</v>
       </c>
     </row>
     <row r="14" spans="1:12" x14ac:dyDescent="0.35">
       <c r="K14" s="11"/>
       <c r="L14" s="12" t="s">
-        <v>368</v>
+        <v>367</v>
       </c>
     </row>
     <row r="15" spans="1:12" x14ac:dyDescent="0.35">
       <c r="K15" s="11"/>
       <c r="L15" s="12" t="s">
-        <v>369</v>
+        <v>368</v>
       </c>
     </row>
     <row r="16" spans="1:12" x14ac:dyDescent="0.35">
       <c r="K16" s="11"/>
       <c r="L16" s="12" t="s">
-        <v>370</v>
+        <v>369</v>
       </c>
     </row>
     <row r="17" spans="11:12" x14ac:dyDescent="0.35">
       <c r="K17" s="11"/>
       <c r="L17" s="12" t="s">
-        <v>371</v>
+        <v>370</v>
       </c>
     </row>
     <row r="18" spans="11:12" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="K18" s="13"/>
       <c r="L18" s="14" t="s">
-        <v>372</v>
+        <v>371</v>
       </c>
     </row>
     <row r="19" spans="11:12" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="K19" s="183" t="s">
-        <v>373</v>
+        <v>372</v>
       </c>
       <c r="L19" s="184"/>
     </row>
@@ -14868,7 +14867,7 @@
       <selection sqref="A1:K1"/>
       <pageMargins left="0" right="0" top="0" bottom="0" header="0" footer="0"/>
       <pageSetup orientation="portrait" r:id="rId1"/>
-      <autoFilter ref="A2:P11" xr:uid="{31D135D1-19CC-4FAC-B376-2E81581D0D4E}"/>
+      <autoFilter ref="A2:P11" xr:uid="{8E9FD0EC-7C93-4FFE-86EC-BEF41D1A6BF2}"/>
     </customSheetView>
   </customSheetViews>
   <mergeCells count="5">
@@ -14913,7 +14912,7 @@
     </row>
     <row r="2" spans="1:9" ht="18.649999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B2" s="187" t="s">
-        <v>374</v>
+        <v>373</v>
       </c>
       <c r="C2" s="188"/>
       <c r="D2" s="173"/>
@@ -14929,7 +14928,7 @@
     </row>
     <row r="4" spans="1:9" ht="18.649999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A4" s="181" t="s">
-        <v>375</v>
+        <v>374</v>
       </c>
       <c r="B4" s="181"/>
       <c r="C4" s="181"/>
@@ -14942,7 +14941,7 @@
     </row>
     <row r="5" spans="1:9" ht="33.65" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A5" s="185" t="s">
-        <v>376</v>
+        <v>375</v>
       </c>
       <c r="B5" s="186"/>
       <c r="C5" s="186"/>
@@ -14983,51 +14982,51 @@
     </row>
     <row r="7" spans="1:9" s="35" customFormat="1" ht="58" x14ac:dyDescent="0.35">
       <c r="A7" s="6" t="s">
+        <v>376</v>
+      </c>
+      <c r="B7" s="8" t="s">
         <v>377</v>
       </c>
-      <c r="B7" s="8" t="s">
+      <c r="C7" s="8" t="s">
         <v>378</v>
-      </c>
-      <c r="C7" s="8" t="s">
-        <v>379</v>
       </c>
       <c r="D7" s="6" t="s">
         <v>235</v>
       </c>
       <c r="E7" s="6" t="s">
+        <v>379</v>
+      </c>
+      <c r="F7" s="6" t="s">
         <v>380</v>
       </c>
-      <c r="F7" s="6" t="s">
+      <c r="G7" s="8" t="s">
         <v>381</v>
-      </c>
-      <c r="G7" s="8" t="s">
-        <v>382</v>
       </c>
       <c r="H7" s="8" t="s">
         <v>308</v>
       </c>
       <c r="I7" s="74" t="s">
-        <v>383</v>
+        <v>382</v>
       </c>
     </row>
     <row r="8" spans="1:9" s="35" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A8" s="6" t="s">
+        <v>383</v>
+      </c>
+      <c r="B8" s="8" t="s">
         <v>384</v>
       </c>
-      <c r="B8" s="8" t="s">
+      <c r="C8" s="8" t="s">
         <v>385</v>
-      </c>
-      <c r="C8" s="8" t="s">
-        <v>386</v>
       </c>
       <c r="D8" s="6" t="s">
         <v>235</v>
       </c>
       <c r="E8" s="6" t="s">
-        <v>380</v>
+        <v>379</v>
       </c>
       <c r="F8" s="6" t="s">
-        <v>387</v>
+        <v>386</v>
       </c>
       <c r="G8" s="6" t="s">
         <v>312</v>
@@ -15039,25 +15038,25 @@
     </row>
     <row r="9" spans="1:9" s="35" customFormat="1" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A9" s="6" t="s">
-        <v>388</v>
+        <v>387</v>
       </c>
       <c r="B9" s="131" t="s">
         <v>238</v>
       </c>
       <c r="C9" s="8" t="s">
-        <v>389</v>
+        <v>388</v>
       </c>
       <c r="D9" s="6" t="s">
         <v>235</v>
       </c>
       <c r="E9" s="6" t="s">
+        <v>389</v>
+      </c>
+      <c r="F9" s="6" t="s">
         <v>390</v>
       </c>
-      <c r="F9" s="6" t="s">
+      <c r="G9" s="8" t="s">
         <v>391</v>
-      </c>
-      <c r="G9" s="8" t="s">
-        <v>392</v>
       </c>
       <c r="H9" s="8" t="s">
         <v>308</v>
@@ -15066,20 +15065,20 @@
     </row>
     <row r="10" spans="1:9" s="35" customFormat="1" ht="58" x14ac:dyDescent="0.35">
       <c r="A10" s="6" t="s">
-        <v>393</v>
+        <v>392</v>
       </c>
       <c r="B10" s="131" t="s">
         <v>183</v>
       </c>
       <c r="C10" s="8" t="s">
-        <v>394</v>
+        <v>393</v>
       </c>
       <c r="D10" s="6"/>
       <c r="E10" s="6" t="s">
-        <v>380</v>
+        <v>379</v>
       </c>
       <c r="F10" s="6" t="s">
-        <v>395</v>
+        <v>394</v>
       </c>
       <c r="G10" s="6" t="s">
         <v>312</v>
@@ -15091,13 +15090,13 @@
     </row>
     <row r="11" spans="1:9" s="35" customFormat="1" ht="29" x14ac:dyDescent="0.35">
       <c r="A11" s="6" t="s">
+        <v>395</v>
+      </c>
+      <c r="B11" s="131" t="s">
         <v>396</v>
       </c>
-      <c r="B11" s="131" t="s">
+      <c r="C11" s="6" t="s">
         <v>397</v>
-      </c>
-      <c r="C11" s="6" t="s">
-        <v>398</v>
       </c>
       <c r="D11" s="6" t="s">
         <v>235</v>
@@ -15118,22 +15117,22 @@
     </row>
     <row r="12" spans="1:9" s="35" customFormat="1" ht="145" x14ac:dyDescent="0.35">
       <c r="A12" s="6" t="s">
+        <v>398</v>
+      </c>
+      <c r="B12" s="131" t="s">
         <v>399</v>
       </c>
-      <c r="B12" s="131" t="s">
+      <c r="C12" s="8" t="s">
         <v>400</v>
-      </c>
-      <c r="C12" s="8" t="s">
-        <v>401</v>
       </c>
       <c r="D12" s="6" t="s">
         <v>235</v>
       </c>
       <c r="E12" s="6" t="s">
-        <v>380</v>
+        <v>379</v>
       </c>
       <c r="F12" s="6" t="s">
-        <v>402</v>
+        <v>401</v>
       </c>
       <c r="G12" s="6" t="s">
         <v>312</v>
@@ -15145,20 +15144,20 @@
     </row>
     <row r="13" spans="1:9" s="35" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A13" s="6" t="s">
+        <v>402</v>
+      </c>
+      <c r="B13" s="131" t="s">
         <v>403</v>
-      </c>
-      <c r="B13" s="131" t="s">
-        <v>404</v>
       </c>
       <c r="C13" s="8"/>
       <c r="D13" s="6" t="s">
         <v>235</v>
       </c>
       <c r="E13" s="6" t="s">
-        <v>380</v>
+        <v>379</v>
       </c>
       <c r="F13" s="6" t="s">
-        <v>405</v>
+        <v>404</v>
       </c>
       <c r="G13" s="6" t="s">
         <v>312</v>
@@ -15170,20 +15169,20 @@
     </row>
     <row r="14" spans="1:9" s="35" customFormat="1" ht="29" x14ac:dyDescent="0.35">
       <c r="A14" s="6" t="s">
+        <v>405</v>
+      </c>
+      <c r="B14" s="131" t="s">
         <v>406</v>
-      </c>
-      <c r="B14" s="131" t="s">
-        <v>407</v>
       </c>
       <c r="C14" s="8"/>
       <c r="D14" s="6" t="s">
         <v>235</v>
       </c>
       <c r="E14" s="6" t="s">
-        <v>380</v>
+        <v>379</v>
       </c>
       <c r="F14" s="6" t="s">
-        <v>408</v>
+        <v>407</v>
       </c>
       <c r="G14" s="6" t="s">
         <v>312</v>
@@ -15195,7 +15194,7 @@
     </row>
     <row r="15" spans="1:9" s="35" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A15" s="6" t="s">
-        <v>409</v>
+        <v>408</v>
       </c>
       <c r="B15" s="131" t="s">
         <v>184</v>
@@ -15205,10 +15204,10 @@
         <v>235</v>
       </c>
       <c r="E15" s="6" t="s">
-        <v>380</v>
+        <v>379</v>
       </c>
       <c r="F15" s="128" t="s">
-        <v>410</v>
+        <v>409</v>
       </c>
       <c r="G15" s="6" t="s">
         <v>312</v>
@@ -15220,20 +15219,20 @@
     </row>
     <row r="16" spans="1:9" s="35" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A16" s="6" t="s">
+        <v>410</v>
+      </c>
+      <c r="B16" s="131" t="s">
         <v>411</v>
-      </c>
-      <c r="B16" s="131" t="s">
-        <v>412</v>
       </c>
       <c r="C16" s="8"/>
       <c r="D16" s="6" t="s">
         <v>235</v>
       </c>
       <c r="E16" s="6" t="s">
-        <v>380</v>
+        <v>379</v>
       </c>
       <c r="F16" s="128" t="s">
-        <v>413</v>
+        <v>412</v>
       </c>
       <c r="G16" s="6" t="s">
         <v>312</v>
@@ -15245,20 +15244,20 @@
     </row>
     <row r="17" spans="1:9" s="35" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A17" s="6" t="s">
+        <v>413</v>
+      </c>
+      <c r="B17" s="8" t="s">
         <v>414</v>
-      </c>
-      <c r="B17" s="8" t="s">
-        <v>415</v>
       </c>
       <c r="C17" s="8"/>
       <c r="D17" s="6" t="s">
         <v>235</v>
       </c>
       <c r="E17" s="6" t="s">
-        <v>380</v>
+        <v>379</v>
       </c>
       <c r="F17" s="6" t="s">
-        <v>416</v>
+        <v>415</v>
       </c>
       <c r="G17" s="6" t="s">
         <v>312</v>
@@ -15270,20 +15269,20 @@
     </row>
     <row r="18" spans="1:9" s="35" customFormat="1" ht="29" x14ac:dyDescent="0.35">
       <c r="A18" s="6" t="s">
+        <v>416</v>
+      </c>
+      <c r="B18" s="8" t="s">
         <v>417</v>
-      </c>
-      <c r="B18" s="8" t="s">
-        <v>418</v>
       </c>
       <c r="C18" s="8"/>
       <c r="D18" s="6" t="s">
         <v>235</v>
       </c>
       <c r="E18" s="6" t="s">
-        <v>380</v>
+        <v>379</v>
       </c>
       <c r="F18" s="6" t="s">
-        <v>419</v>
+        <v>418</v>
       </c>
       <c r="G18" s="6" t="s">
         <v>312</v>
@@ -15295,7 +15294,7 @@
     </row>
     <row r="19" spans="1:9" s="35" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A19" s="6" t="s">
-        <v>420</v>
+        <v>419</v>
       </c>
       <c r="B19" s="8" t="s">
         <v>185</v>
@@ -15305,10 +15304,10 @@
         <v>235</v>
       </c>
       <c r="E19" s="6" t="s">
-        <v>380</v>
+        <v>379</v>
       </c>
       <c r="F19" s="6" t="s">
-        <v>421</v>
+        <v>420</v>
       </c>
       <c r="G19" s="6" t="s">
         <v>312</v>
@@ -15320,20 +15319,20 @@
     </row>
     <row r="20" spans="1:9" s="35" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A20" s="6" t="s">
+        <v>421</v>
+      </c>
+      <c r="B20" s="8" t="s">
         <v>422</v>
-      </c>
-      <c r="B20" s="8" t="s">
-        <v>423</v>
       </c>
       <c r="C20" s="8"/>
       <c r="D20" s="6" t="s">
         <v>235</v>
       </c>
       <c r="E20" s="6" t="s">
-        <v>380</v>
+        <v>379</v>
       </c>
       <c r="F20" s="6" t="s">
-        <v>424</v>
+        <v>423</v>
       </c>
       <c r="G20" s="6" t="s">
         <v>312</v>
@@ -15345,7 +15344,7 @@
     </row>
     <row r="21" spans="1:9" s="35" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A21" s="6" t="s">
-        <v>425</v>
+        <v>424</v>
       </c>
       <c r="B21" s="8" t="s">
         <v>76</v>
@@ -15355,10 +15354,10 @@
         <v>235</v>
       </c>
       <c r="E21" s="6" t="s">
+        <v>425</v>
+      </c>
+      <c r="F21" s="6" t="s">
         <v>426</v>
-      </c>
-      <c r="F21" s="6" t="s">
-        <v>427</v>
       </c>
       <c r="G21" s="6" t="s">
         <v>312</v>
@@ -15370,7 +15369,7 @@
     </row>
     <row r="22" spans="1:9" s="35" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A22" s="6" t="s">
-        <v>428</v>
+        <v>427</v>
       </c>
       <c r="B22" s="8" t="s">
         <v>78</v>
@@ -15380,7 +15379,7 @@
         <v>235</v>
       </c>
       <c r="E22" s="6" t="s">
-        <v>429</v>
+        <v>428</v>
       </c>
       <c r="F22" s="6" t="s">
         <v>347</v>
@@ -15395,7 +15394,7 @@
     </row>
     <row r="23" spans="1:9" s="35" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A23" s="6" t="s">
-        <v>430</v>
+        <v>429</v>
       </c>
       <c r="B23" s="8" t="s">
         <v>186</v>
@@ -15405,10 +15404,10 @@
         <v>235</v>
       </c>
       <c r="E23" s="6" t="s">
-        <v>380</v>
+        <v>379</v>
       </c>
       <c r="F23" s="6" t="s">
-        <v>431</v>
+        <v>430</v>
       </c>
       <c r="G23" s="6" t="s">
         <v>312</v>
@@ -15420,20 +15419,20 @@
     </row>
     <row r="24" spans="1:9" s="35" customFormat="1" ht="29" x14ac:dyDescent="0.35">
       <c r="A24" s="6" t="s">
+        <v>431</v>
+      </c>
+      <c r="B24" s="8" t="s">
         <v>432</v>
-      </c>
-      <c r="B24" s="8" t="s">
-        <v>433</v>
       </c>
       <c r="C24" s="8"/>
       <c r="D24" s="6" t="s">
         <v>235</v>
       </c>
       <c r="E24" s="6" t="s">
-        <v>380</v>
+        <v>379</v>
       </c>
       <c r="F24" s="6" t="s">
-        <v>434</v>
+        <v>433</v>
       </c>
       <c r="G24" s="6" t="s">
         <v>312</v>
@@ -15445,7 +15444,7 @@
     </row>
     <row r="25" spans="1:9" s="35" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A25" s="6" t="s">
-        <v>435</v>
+        <v>434</v>
       </c>
       <c r="B25" s="8" t="s">
         <v>187</v>
@@ -15455,10 +15454,10 @@
         <v>235</v>
       </c>
       <c r="E25" s="6" t="s">
-        <v>380</v>
+        <v>379</v>
       </c>
       <c r="F25" s="6" t="s">
-        <v>436</v>
+        <v>435</v>
       </c>
       <c r="G25" s="6" t="s">
         <v>312</v>
@@ -15470,20 +15469,20 @@
     </row>
     <row r="26" spans="1:9" s="35" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A26" s="6" t="s">
+        <v>436</v>
+      </c>
+      <c r="B26" s="8" t="s">
         <v>437</v>
-      </c>
-      <c r="B26" s="8" t="s">
-        <v>438</v>
       </c>
       <c r="C26" s="8"/>
       <c r="D26" s="6" t="s">
         <v>235</v>
       </c>
       <c r="E26" s="6" t="s">
-        <v>380</v>
+        <v>379</v>
       </c>
       <c r="F26" s="6" t="s">
-        <v>439</v>
+        <v>438</v>
       </c>
       <c r="G26" s="6" t="s">
         <v>312</v>
@@ -15495,7 +15494,7 @@
     </row>
     <row r="27" spans="1:9" s="35" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A27" s="6" t="s">
-        <v>440</v>
+        <v>439</v>
       </c>
       <c r="B27" s="8" t="s">
         <v>188</v>
@@ -15505,10 +15504,10 @@
         <v>235</v>
       </c>
       <c r="E27" s="6" t="s">
-        <v>380</v>
+        <v>379</v>
       </c>
       <c r="F27" s="6" t="s">
-        <v>441</v>
+        <v>440</v>
       </c>
       <c r="G27" s="6" t="s">
         <v>312</v>
@@ -15520,20 +15519,20 @@
     </row>
     <row r="28" spans="1:9" s="35" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A28" s="6" t="s">
+        <v>441</v>
+      </c>
+      <c r="B28" s="8" t="s">
         <v>442</v>
-      </c>
-      <c r="B28" s="8" t="s">
-        <v>443</v>
       </c>
       <c r="C28" s="8"/>
       <c r="D28" s="6" t="s">
         <v>235</v>
       </c>
       <c r="E28" s="6" t="s">
-        <v>380</v>
+        <v>379</v>
       </c>
       <c r="F28" s="6" t="s">
-        <v>444</v>
+        <v>443</v>
       </c>
       <c r="G28" s="6" t="s">
         <v>312</v>
@@ -15545,7 +15544,7 @@
     </row>
     <row r="29" spans="1:9" s="35" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A29" s="6" t="s">
-        <v>445</v>
+        <v>444</v>
       </c>
       <c r="B29" s="8" t="s">
         <v>189</v>
@@ -15555,10 +15554,10 @@
         <v>235</v>
       </c>
       <c r="E29" s="6" t="s">
-        <v>380</v>
+        <v>379</v>
       </c>
       <c r="F29" s="6" t="s">
-        <v>446</v>
+        <v>445</v>
       </c>
       <c r="G29" s="6" t="s">
         <v>312</v>
@@ -15570,20 +15569,20 @@
     </row>
     <row r="30" spans="1:9" s="35" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A30" s="6" t="s">
+        <v>446</v>
+      </c>
+      <c r="B30" s="8" t="s">
         <v>447</v>
-      </c>
-      <c r="B30" s="8" t="s">
-        <v>448</v>
       </c>
       <c r="C30" s="8"/>
       <c r="D30" s="6" t="s">
         <v>235</v>
       </c>
       <c r="E30" s="6" t="s">
-        <v>380</v>
+        <v>379</v>
       </c>
       <c r="F30" s="6" t="s">
-        <v>449</v>
+        <v>448</v>
       </c>
       <c r="G30" s="6" t="s">
         <v>312</v>
@@ -15595,7 +15594,7 @@
     </row>
     <row r="31" spans="1:9" s="35" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A31" s="6" t="s">
-        <v>450</v>
+        <v>449</v>
       </c>
       <c r="B31" s="8" t="s">
         <v>190</v>
@@ -15605,10 +15604,10 @@
         <v>235</v>
       </c>
       <c r="E31" s="6" t="s">
-        <v>380</v>
+        <v>379</v>
       </c>
       <c r="F31" s="6" t="s">
-        <v>451</v>
+        <v>450</v>
       </c>
       <c r="G31" s="6" t="s">
         <v>312</v>
@@ -15620,20 +15619,20 @@
     </row>
     <row r="32" spans="1:9" s="35" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A32" s="6" t="s">
+        <v>451</v>
+      </c>
+      <c r="B32" s="8" t="s">
         <v>452</v>
-      </c>
-      <c r="B32" s="8" t="s">
-        <v>453</v>
       </c>
       <c r="C32" s="8"/>
       <c r="D32" s="6" t="s">
         <v>235</v>
       </c>
       <c r="E32" s="6" t="s">
-        <v>380</v>
+        <v>379</v>
       </c>
       <c r="F32" s="6" t="s">
-        <v>454</v>
+        <v>453</v>
       </c>
       <c r="G32" s="6" t="s">
         <v>312</v>
@@ -15645,20 +15644,20 @@
     </row>
     <row r="33" spans="1:9" s="35" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A33" s="6" t="s">
+        <v>454</v>
+      </c>
+      <c r="B33" s="8" t="s">
         <v>455</v>
-      </c>
-      <c r="B33" s="8" t="s">
-        <v>456</v>
       </c>
       <c r="C33" s="8"/>
       <c r="D33" s="6" t="s">
         <v>235</v>
       </c>
       <c r="E33" s="6" t="s">
-        <v>380</v>
+        <v>379</v>
       </c>
       <c r="F33" s="6" t="s">
-        <v>456</v>
+        <v>455</v>
       </c>
       <c r="G33" s="6" t="s">
         <v>312</v>
@@ -15727,7 +15726,7 @@
     </row>
     <row r="2" spans="1:7" ht="41.15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A2" s="182" t="s">
-        <v>457</v>
+        <v>456</v>
       </c>
       <c r="B2" s="182"/>
       <c r="C2" s="170"/>
@@ -15771,22 +15770,22 @@
         <v>182</v>
       </c>
       <c r="B5" s="8" t="s">
-        <v>458</v>
+        <v>457</v>
       </c>
       <c r="C5" s="66" t="s">
         <v>235</v>
       </c>
       <c r="D5" s="66" t="s">
+        <v>458</v>
+      </c>
+      <c r="E5" s="67" t="s">
         <v>459</v>
       </c>
-      <c r="E5" s="67" t="s">
+      <c r="F5" s="58" t="s">
         <v>460</v>
       </c>
-      <c r="F5" s="58" t="s">
-        <v>461</v>
-      </c>
       <c r="G5" s="58" t="s">
-        <v>461</v>
+        <v>460</v>
       </c>
     </row>
     <row r="6" spans="1:7" ht="29" x14ac:dyDescent="0.35">
@@ -15794,22 +15793,22 @@
         <v>12</v>
       </c>
       <c r="B6" s="8" t="s">
-        <v>462</v>
+        <v>461</v>
       </c>
       <c r="C6" s="66" t="s">
         <v>235</v>
       </c>
       <c r="D6" s="66" t="s">
+        <v>462</v>
+      </c>
+      <c r="E6" s="104" t="s">
         <v>463</v>
       </c>
-      <c r="E6" s="104" t="s">
-        <v>464</v>
-      </c>
       <c r="F6" s="58" t="s">
-        <v>461</v>
+        <v>460</v>
       </c>
       <c r="G6" s="58" t="s">
-        <v>461</v>
+        <v>460</v>
       </c>
     </row>
     <row r="7" spans="1:7" ht="29" x14ac:dyDescent="0.35">
@@ -15823,24 +15822,24 @@
         <v>235</v>
       </c>
       <c r="D7" s="66" t="s">
-        <v>463</v>
+        <v>462</v>
       </c>
       <c r="E7" s="104" t="s">
-        <v>465</v>
+        <v>464</v>
       </c>
       <c r="F7" s="58" t="s">
-        <v>461</v>
+        <v>460</v>
       </c>
       <c r="G7" s="58" t="s">
-        <v>461</v>
+        <v>460</v>
       </c>
     </row>
     <row r="8" spans="1:7" ht="101.5" x14ac:dyDescent="0.35">
       <c r="A8" s="8" t="s">
+        <v>465</v>
+      </c>
+      <c r="B8" s="8" t="s">
         <v>466</v>
-      </c>
-      <c r="B8" s="8" t="s">
-        <v>467</v>
       </c>
       <c r="C8" s="66" t="s">
         <v>235</v>
@@ -15849,13 +15848,13 @@
         <v>82</v>
       </c>
       <c r="E8" s="66" t="s">
-        <v>468</v>
+        <v>467</v>
       </c>
       <c r="F8" s="58" t="s">
-        <v>461</v>
+        <v>460</v>
       </c>
       <c r="G8" s="58" t="s">
-        <v>461</v>
+        <v>460</v>
       </c>
     </row>
     <row r="9" spans="1:7" ht="87" x14ac:dyDescent="0.35">
@@ -15863,7 +15862,7 @@
         <v>26</v>
       </c>
       <c r="B9" s="8" t="s">
-        <v>469</v>
+        <v>468</v>
       </c>
       <c r="C9" s="66"/>
       <c r="D9" s="66" t="s">
@@ -15873,10 +15872,10 @@
         <v>274</v>
       </c>
       <c r="F9" s="58" t="s">
-        <v>461</v>
+        <v>460</v>
       </c>
       <c r="G9" s="58" t="s">
-        <v>461</v>
+        <v>460</v>
       </c>
     </row>
   </sheetData>
@@ -15924,7 +15923,7 @@
     </row>
     <row r="2" spans="1:32" x14ac:dyDescent="0.35">
       <c r="B2" s="182" t="s">
-        <v>470</v>
+        <v>469</v>
       </c>
       <c r="C2" s="182"/>
       <c r="D2" s="173"/>
@@ -15947,7 +15946,7 @@
     </row>
     <row r="5" spans="1:32" x14ac:dyDescent="0.35">
       <c r="A5" s="181" t="s">
-        <v>471</v>
+        <v>470</v>
       </c>
       <c r="B5" s="181"/>
       <c r="C5" s="181"/>
@@ -15959,7 +15958,7 @@
     </row>
     <row r="6" spans="1:32" ht="41.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A6" s="186" t="s">
-        <v>472</v>
+        <v>471</v>
       </c>
       <c r="B6" s="186"/>
       <c r="C6" s="186"/>
@@ -15969,10 +15968,10 @@
       <c r="G6" s="186"/>
       <c r="H6" s="186"/>
       <c r="AA6" t="s">
+        <v>472</v>
+      </c>
+      <c r="AB6" s="192" t="s">
         <v>473</v>
-      </c>
-      <c r="AB6" s="192" t="s">
-        <v>474</v>
       </c>
       <c r="AC6" s="192"/>
       <c r="AD6" s="192"/>
@@ -16008,45 +16007,45 @@
         <v>167</v>
       </c>
       <c r="Y7" s="111" t="s">
+        <v>474</v>
+      </c>
+      <c r="Z7" s="111" t="s">
         <v>475</v>
       </c>
-      <c r="Z7" s="111" t="s">
+      <c r="AA7" s="64" t="s">
         <v>476</v>
       </c>
-      <c r="AA7" s="64" t="s">
+      <c r="AB7" s="64" t="s">
         <v>477</v>
       </c>
-      <c r="AB7" s="64" t="s">
+      <c r="AC7" s="64" t="s">
         <v>478</v>
       </c>
-      <c r="AC7" s="64" t="s">
+      <c r="AD7" s="64" t="s">
         <v>479</v>
-      </c>
-      <c r="AD7" s="64" t="s">
-        <v>480</v>
       </c>
     </row>
     <row r="8" spans="1:32" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A8" s="6" t="s">
-        <v>481</v>
+        <v>480</v>
       </c>
       <c r="B8" s="120" t="s">
         <v>174</v>
       </c>
       <c r="C8" s="6" t="s">
-        <v>482</v>
+        <v>481</v>
       </c>
       <c r="D8" s="6" t="s">
         <v>235</v>
       </c>
       <c r="E8" s="6" t="s">
-        <v>483</v>
+        <v>482</v>
       </c>
       <c r="F8" s="6" t="s">
         <v>276</v>
       </c>
       <c r="G8" s="24" t="s">
-        <v>484</v>
+        <v>483</v>
       </c>
       <c r="H8" s="24" t="s">
         <v>308</v>
@@ -16055,25 +16054,25 @@
     </row>
     <row r="9" spans="1:32" ht="29" x14ac:dyDescent="0.35">
       <c r="A9" s="6" t="s">
-        <v>485</v>
+        <v>484</v>
       </c>
       <c r="B9" s="6" t="s">
         <v>238</v>
       </c>
       <c r="C9" s="6" t="s">
-        <v>486</v>
+        <v>485</v>
       </c>
       <c r="D9" s="6" t="s">
         <v>235</v>
       </c>
       <c r="E9" s="6" t="s">
-        <v>487</v>
+        <v>486</v>
       </c>
       <c r="F9" s="6" t="s">
         <v>43</v>
       </c>
       <c r="G9" s="24" t="s">
-        <v>488</v>
+        <v>487</v>
       </c>
       <c r="H9" s="24" t="s">
         <v>308</v>
@@ -16082,13 +16081,13 @@
     </row>
     <row r="10" spans="1:32" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A10" s="6" t="s">
-        <v>489</v>
+        <v>488</v>
       </c>
       <c r="B10" s="120" t="s">
         <v>254</v>
       </c>
       <c r="C10" s="8" t="s">
-        <v>490</v>
+        <v>489</v>
       </c>
       <c r="D10" s="6" t="s">
         <v>235</v>
@@ -16100,34 +16099,34 @@
         <v>256</v>
       </c>
       <c r="G10" s="24" t="s">
-        <v>491</v>
+        <v>490</v>
       </c>
       <c r="H10" s="24" t="s">
         <v>308</v>
       </c>
       <c r="I10" s="3"/>
       <c r="J10" s="115" t="s">
-        <v>492</v>
+        <v>491</v>
       </c>
     </row>
     <row r="11" spans="1:32" ht="72.5" x14ac:dyDescent="0.35">
       <c r="A11" s="6" t="s">
+        <v>492</v>
+      </c>
+      <c r="B11" s="6" t="s">
         <v>493</v>
       </c>
-      <c r="B11" s="6" t="s">
+      <c r="C11" s="8" t="s">
         <v>494</v>
-      </c>
-      <c r="C11" s="8" t="s">
-        <v>495</v>
       </c>
       <c r="D11" s="6" t="s">
         <v>235</v>
       </c>
       <c r="E11" s="6" t="s">
-        <v>483</v>
+        <v>482</v>
       </c>
       <c r="F11" s="8" t="s">
-        <v>496</v>
+        <v>495</v>
       </c>
       <c r="G11" s="6" t="s">
         <v>312</v>

</xml_diff>